<commit_message>
Corrige les plages de formules du tableau de bord
Les references vers l'onglet Inventaire etaient malformees : la lettre de
colonne manquait apres le deux-points, produisant des plages du type
Inventaire!A2:401 au lieu de Inventaire!$A$2:$A$401. Les 20 formules du
tableau de bord (COUNTA, SUM, COUNTIFS, SUMIFS) auraient renvoye une
erreur a l'ouverture du classeur.

Ajoute un helper rg() qui construit la plage absolue d'une colonne, et
verifie par script que les 20 plages sont desormais bien formees.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013W9yFMU4pNLbCpPtWZwhqw
</commit_message>
<xml_diff>
--- a/lithographies/inventaire-lithographies.xlsx
+++ b/lithographies/inventaire-lithographies.xlsx
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="C5" s="9">
-        <f>COUNTA(Inventaire!A2:401)</f>
+        <f>COUNTA(Inventaire!$A$2:$A$401)</f>
         <v/>
       </c>
     </row>
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="C6" s="9">
-        <f>SUM(Inventaire!O2:401)</f>
+        <f>SUM(Inventaire!$O$2:$O$401)</f>
         <v/>
       </c>
     </row>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="C7" s="9">
-        <f>COUNTIFS(Inventaire!Q2:401,"Oui")</f>
+        <f>COUNTIFS(Inventaire!$Q$2:$Q$401,"Oui")</f>
         <v/>
       </c>
     </row>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="C8" s="9">
-        <f>COUNTIFS(Inventaire!R2:401,"Oui — litho")</f>
+        <f>COUNTIFS(Inventaire!$R$2:$R$401,"Oui — litho")</f>
         <v/>
       </c>
     </row>
@@ -961,15 +961,15 @@
         </is>
       </c>
       <c r="C11" s="11">
-        <f>COUNTIFS(Inventaire!S2:401,"A")</f>
+        <f>COUNTIFS(Inventaire!$S$2:$S$401,"A")</f>
         <v/>
       </c>
       <c r="D11" s="11">
-        <f>SUMIFS(Inventaire!O2:401,Inventaire!S2:401,"A")</f>
+        <f>SUMIFS(Inventaire!$O$2:$O$401,Inventaire!$S$2:$S$401,"A")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>SUMIFS(Inventaire!V2:401,Inventaire!S2:401,"A")</f>
+        <f>SUMIFS(Inventaire!$V$2:$V$401,Inventaire!$S$2:$S$401,"A")</f>
         <v/>
       </c>
     </row>
@@ -980,15 +980,15 @@
         </is>
       </c>
       <c r="C12" s="11">
-        <f>COUNTIFS(Inventaire!S2:401,"B")</f>
+        <f>COUNTIFS(Inventaire!$S$2:$S$401,"B")</f>
         <v/>
       </c>
       <c r="D12" s="11">
-        <f>SUMIFS(Inventaire!O2:401,Inventaire!S2:401,"B")</f>
+        <f>SUMIFS(Inventaire!$O$2:$O$401,Inventaire!$S$2:$S$401,"B")</f>
         <v/>
       </c>
       <c r="E12" s="12">
-        <f>SUMIFS(Inventaire!V2:401,Inventaire!S2:401,"B")</f>
+        <f>SUMIFS(Inventaire!$V$2:$V$401,Inventaire!$S$2:$S$401,"B")</f>
         <v/>
       </c>
     </row>
@@ -999,15 +999,15 @@
         </is>
       </c>
       <c r="C13" s="11">
-        <f>COUNTIFS(Inventaire!S2:401,"C")</f>
+        <f>COUNTIFS(Inventaire!$S$2:$S$401,"C")</f>
         <v/>
       </c>
       <c r="D13" s="11">
-        <f>SUMIFS(Inventaire!O2:401,Inventaire!S2:401,"C")</f>
+        <f>SUMIFS(Inventaire!$O$2:$O$401,Inventaire!$S$2:$S$401,"C")</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>SUMIFS(Inventaire!V2:401,Inventaire!S2:401,"C")</f>
+        <f>SUMIFS(Inventaire!$V$2:$V$401,Inventaire!$S$2:$S$401,"C")</f>
         <v/>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="C17" s="9">
-        <f>COUNTIFS(Inventaire!X2:401,"En ligne")</f>
+        <f>COUNTIFS(Inventaire!$X$2:$X$401,"En ligne")</f>
         <v/>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="C18" s="9">
-        <f>COUNTIFS(Inventaire!X2:401,"VENDUE")</f>
+        <f>COUNTIFS(Inventaire!$X$2:$X$401,"VENDUE")</f>
         <v/>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="C19" s="9">
-        <f>COUNTIFS(Inventaire!X2:401,"Invendue")+COUNTIFS(Inventaire!X2:401,"Retirée")</f>
+        <f>COUNTIFS(Inventaire!$X$2:$X$401,"Invendue")+COUNTIFS(Inventaire!$X$2:$X$401,"Retirée")</f>
         <v/>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="C22" s="16">
-        <f>SUM(Inventaire!Z2:401)</f>
+        <f>SUM(Inventaire!$Z$2:$Z$401)</f>
         <v/>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="C23" s="16">
-        <f>SUM(Inventaire!AA2:401)</f>
+        <f>SUM(Inventaire!$AA$2:$AA$401)</f>
         <v/>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="C24" s="17">
-        <f>SUM(Inventaire!AB2:401)</f>
+        <f>SUM(Inventaire!$AB$2:$AB$401)</f>
         <v/>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="C25" s="16">
-        <f>IFERROR(SUM(Inventaire!AB2:401)/COUNTIFS(Inventaire!X2:401,"VENDUE"),0)</f>
+        <f>IFERROR(SUM(Inventaire!$AB$2:$AB$401)/COUNTIFS(Inventaire!$X$2:$X$401,"VENDUE"),0)</f>
         <v/>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="C29" s="9">
-        <f>COUNTIFS(Inventaire!Z2:401,"&gt;5000")</f>
+        <f>COUNTIFS(Inventaire!$Z$2:$Z$401,"&gt;5000")</f>
         <v/>
       </c>
       <c r="G29" s="19" t="inlineStr">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="C30" s="9">
-        <f>COUNTIFS(Inventaire!X2:401,"VENDUE")</f>
+        <f>COUNTIFS(Inventaire!$X$2:$X$401,"VENDUE")</f>
         <v/>
       </c>
       <c r="G30" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Etend les reperes de prix aux cinq artistes identifies
Ajoute Yves Brayer, Camille Hilaire et Hasegawa aux cotes deja relevees
pour Toffoli et Weisbuch, et restructure l'onglet en cinq sections :

- hierarchie des artistes par priorite de vente, avec fourchette nette
- 15 prix observes, en distinguant adjuge (fond vert) de demande (rose)
- mise au point sur Artprice : base de donnees payante, pas un canal de
  vente, avec les alternatives gratuites
- citations d'experts et facteurs de valorisation par artiste

Signale la confusion possible entre Kiyoshi Hasegawa (1891-1980, maniere
noire, cote elevee) et Shoichi Hasegawa (1929-2023).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013W9yFMU4pNLbCpPtWZwhqw
</commit_message>
<xml_diff>
--- a/lithographies/inventaire-lithographies.xlsx
+++ b/lithographies/inventaire-lithographies.xlsx
@@ -74,7 +74,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +104,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -138,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -200,26 +205,38 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -16920,363 +16937,859 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G25"/>
+  <dimension ref="B1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Repères de prix observés</t>
+          <t>Repères de prix — 5 artistes identifiés</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="19" t="inlineStr">
         <is>
-          <t>Distinction capitale : un PRIX DEMANDÉ n'est pas un PRIX OBTENU. Les galeries affichent 400-1 200 € ; les enchères adjugent 50-250 €.</t>
+          <t>Règle n°1 : un PRIX DEMANDÉ n'est pas un PRIX OBTENU. Les galeries affichent 400-1 200 €, les salles adjugent 50-550 €. Cale-toi sur la colonne ADJUGÉ.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Hiérarchie de tes artistes — par où commencer</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="8" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>Artiste</t>
         </is>
       </c>
-      <c r="C4" s="28" t="inlineStr">
-        <is>
-          <t>Référence observée</t>
-        </is>
-      </c>
-      <c r="D4" s="28" t="inlineStr">
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>Net bas</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>Net haut</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr"/>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>Pourquoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Yves Brayer (1907-1990)</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>1 — LE MEILLEUR</t>
+        </is>
+      </c>
+      <c r="D6" s="31" t="n">
+        <v>150</v>
+      </c>
+      <c r="E6" s="31" t="n">
+        <v>500</v>
+      </c>
+      <c r="F6" s="32" t="inlineStr">
+        <is>
+          <t>Membre de l'Institut, musée à son nom aux Baux. Camargue, taureaux, Provence. Seul de tes artistes dont les lithos passent régulièrement les 500 € en salle.</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="n"/>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Hasegawa</t>
+        </is>
+      </c>
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>2 — À CLARIFIER</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="n">
+        <v>60</v>
+      </c>
+      <c r="E7" s="31" t="n">
+        <v>250</v>
+      </c>
+      <c r="F7" s="32" t="inlineStr">
+        <is>
+          <t>S'il s'agit de KIYOSHI Hasegawa (1891-1980, manière noire), la cote est nettement supérieure. Si c'est SHOICHI (1929-2023), on reste dans la fourchette ci-contre. Vérifie le prénom sur les certificats — l'écart est énorme.</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="n"/>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>Claude Weisbuch (1927-2014)</t>
+        </is>
+      </c>
+      <c r="C8" s="34" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D8" s="31" t="n">
+        <v>60</v>
+      </c>
+      <c r="E8" s="31" t="n">
+        <v>200</v>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>Cavaliers, musiciens, théâtre. Cote en baisse mais les estampes résistent mieux que ses huiles.</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="n"/>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Camille Hilaire (1916-2004)</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D9" s="31" t="n">
+        <v>50</v>
+      </c>
+      <c r="E9" s="31" t="n">
+        <v>150</v>
+      </c>
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>Paysages, forêts, chevaux. Très présent sur le marché, prix courants 89-150 €.</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="n"/>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Louis Toffoli (1907-1999)</t>
+        </is>
+      </c>
+      <c r="C10" s="34" t="inlineStr">
+        <is>
+          <t>5 — LE PLUS COMMUN</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" s="31" t="n">
+        <v>180</v>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
+        <is>
+          <t>Éditions très nombreuses. Sujets musiciens et maternités = le haut de la fourchette ; le reste peine à dépasser 100 €.</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Fourchettes NETTES par pièce, après frais de plateforme — synthèse des résultats observés ci-dessous, pas une cotation officielle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Prix réellement observés, avec sources</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Artiste</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>Référence</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
         <is>
           <t>Type de prix</t>
         </is>
       </c>
-      <c r="E4" s="28" t="inlineStr">
-        <is>
-          <t>Bas (€)</t>
-        </is>
-      </c>
-      <c r="F4" s="28" t="inlineStr">
-        <is>
-          <t>Haut (€)</t>
-        </is>
-      </c>
-      <c r="G4" s="28" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
+        <is>
+          <t>Bas</t>
+        </is>
+      </c>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>Haut</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="29" t="inlineStr">
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>Yves Brayer</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>Scène taurine, litho couleur signée au crayon</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>ADJUGÉ</t>
+        </is>
+      </c>
+      <c r="E15" s="36" t="n">
+        <v>550</v>
+      </c>
+      <c r="F15" s="36" t="n">
+        <v>550</v>
+      </c>
+      <c r="G15" s="35" t="inlineStr">
+        <is>
+          <t>Résultat de salle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>Yves Brayer</t>
+        </is>
+      </c>
+      <c r="C16" s="35" t="inlineStr">
+        <is>
+          <t>Suite de 6 lithographies, Camargue, bon état</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>ADJUGÉ</t>
+        </is>
+      </c>
+      <c r="E16" s="36" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F16" s="36" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G16" s="35" t="inlineStr">
+        <is>
+          <t>Résultat de salle — l'intérêt des séries complètes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>Yves Brayer</t>
+        </is>
+      </c>
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>Lithographies signées et numérotées</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>Fourchette marché</t>
+        </is>
+      </c>
+      <c r="E17" s="37" t="n">
+        <v>200</v>
+      </c>
+      <c r="F17" s="37" t="n">
+        <v>600</v>
+      </c>
+      <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>mr-expert.com / gazette-drouot.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>Shoichi Hasegawa</t>
+        </is>
+      </c>
+      <c r="C18" s="32" t="inlineStr">
+        <is>
+          <t>Estampes et multiples, estimation en salle</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>Fourchette marché</t>
+        </is>
+      </c>
+      <c r="E18" s="37" t="n">
+        <v>40</v>
+      </c>
+      <c r="F18" s="37" t="n">
+        <v>300</v>
+      </c>
+      <c r="G18" s="32" t="inlineStr">
+        <is>
+          <t>mr-expert.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>Shoichi Hasegawa</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>Estampes-multiples selon base Artprice</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>Fourchette base</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="F19" s="37" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>Artprice, via galerie-creation</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>Kiyoshi Hasegawa</t>
+        </is>
+      </c>
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t>À NE PAS CONFONDRE — maître de la manière noire</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>Repère</t>
+        </is>
+      </c>
+      <c r="E20" s="37" t="n">
+        <v>300</v>
+      </c>
+      <c r="F20" s="37" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G20" s="32" t="inlineStr">
+        <is>
+          <t>mr-expert.com — cote très supérieure</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>Claude Weisbuch</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="inlineStr">
+        <is>
+          <t>« Grande parade », litho signée en bas à droite</t>
+        </is>
+      </c>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>Estimation salle (2025)</t>
+        </is>
+      </c>
+      <c r="E21" s="37" t="n">
+        <v>200</v>
+      </c>
+      <c r="F21" s="37" t="n">
+        <v>300</v>
+      </c>
+      <c r="G21" s="32" t="inlineStr">
+        <is>
+          <t>primardeco.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="B22" s="32" t="inlineStr">
+        <is>
+          <t>Claude Weisbuch</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="inlineStr">
+        <is>
+          <t>Multiples, fourchette générale</t>
+        </is>
+      </c>
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <t>Fourchette marché</t>
+        </is>
+      </c>
+      <c r="E22" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="F22" s="37" t="n">
+        <v>400</v>
+      </c>
+      <c r="G22" s="32" t="inlineStr">
+        <is>
+          <t>mr-expert.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="B23" s="38" t="inlineStr">
+        <is>
+          <t>Claude Weisbuch</t>
+        </is>
+      </c>
+      <c r="C23" s="38" t="inlineStr">
+        <is>
+          <t>« Deux Cavaliers », litho signée /125</t>
+        </is>
+      </c>
+      <c r="D23" s="38" t="inlineStr">
+        <is>
+          <t>PRIX DEMANDÉ</t>
+        </is>
+      </c>
+      <c r="E23" s="39" t="n">
+        <v>487</v>
+      </c>
+      <c r="F23" s="39" t="n">
+        <v>487</v>
+      </c>
+      <c r="G23" s="38" t="inlineStr">
+        <is>
+          <t>1stdibs.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>Camille Hilaire</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="inlineStr">
+        <is>
+          <t>Multiples en salle, fourchette générale</t>
+        </is>
+      </c>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>Fourchette marché</t>
+        </is>
+      </c>
+      <c r="E24" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" s="37" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G24" s="32" t="inlineStr">
+        <is>
+          <t>mr-expert.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t>Camille Hilaire</t>
+        </is>
+      </c>
+      <c r="C25" s="38" t="inlineStr">
+        <is>
+          <t>Lithographies signées, prix courants en ligne</t>
+        </is>
+      </c>
+      <c r="D25" s="38" t="inlineStr">
+        <is>
+          <t>PRIX DEMANDÉ</t>
+        </is>
+      </c>
+      <c r="E25" s="39" t="n">
+        <v>89</v>
+      </c>
+      <c r="F25" s="39" t="n">
+        <v>280</v>
+      </c>
+      <c r="G25" s="38" t="inlineStr">
+        <is>
+          <t>leboncoin / passion-estampes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="35" t="inlineStr">
         <is>
           <t>Louis Toffoli</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>« Maternité », litho couleurs 50x65, 53/150</t>
-        </is>
-      </c>
-      <c r="D5" s="29" t="inlineStr">
+      <c r="C26" s="35" t="inlineStr">
+        <is>
+          <t>« Maternité » 50x65, n° 53/150 — estimée 60-80 €</t>
+        </is>
+      </c>
+      <c r="D26" s="35" t="inlineStr">
         <is>
           <t>ADJUGÉ (2021)</t>
         </is>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E26" s="36" t="n">
         <v>100</v>
       </c>
-      <c r="F5" s="30" t="n">
+      <c r="F26" s="36" t="n">
         <v>100</v>
       </c>
-      <c r="G5" s="29" t="inlineStr">
-        <is>
-          <t>mw-encheres.com — estimée 60-80 €, adjugée 100 €</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="31" t="inlineStr">
+      <c r="G26" s="35" t="inlineStr">
+        <is>
+          <t>mw-encheres.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="32" t="inlineStr">
         <is>
           <t>Louis Toffoli</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C27" s="32" t="inlineStr">
         <is>
           <t>« Couple sur un banc », litho sur japon 50x73</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D27" s="32" t="inlineStr">
         <is>
           <t>Estimation salle (2023)</t>
         </is>
       </c>
-      <c r="E6" s="32" t="n">
+      <c r="E27" s="37" t="n">
         <v>50</v>
       </c>
-      <c r="F6" s="32" t="n">
+      <c r="F27" s="37" t="n">
         <v>100</v>
       </c>
-      <c r="G6" s="31" t="inlineStr">
+      <c r="G27" s="32" t="inlineStr">
         <is>
           <t>richardmdv.com, vente du 12/12/2023</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="29" t="inlineStr">
+    <row r="28" ht="26" customHeight="1">
+      <c r="B28" s="32" t="inlineStr">
         <is>
           <t>Louis Toffoli</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>Fourchette générale des estampes en salle</t>
-        </is>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
-        <is>
-          <t>Adjugé (marché)</t>
-        </is>
-      </c>
-      <c r="E7" s="30" t="n">
+      <c r="C28" s="32" t="inlineStr">
+        <is>
+          <t>Estampes, fourchette générale en salle</t>
+        </is>
+      </c>
+      <c r="D28" s="32" t="inlineStr">
+        <is>
+          <t>Fourchette marché</t>
+        </is>
+      </c>
+      <c r="E28" s="37" t="n">
         <v>30</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F28" s="37" t="n">
         <v>300</v>
       </c>
-      <c r="G7" s="29" t="inlineStr">
+      <c r="G28" s="32" t="inlineStr">
         <is>
           <t>mr-expert.com / expertisez.com</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="B8" s="33" t="inlineStr">
+    <row r="29" ht="26" customHeight="1">
+      <c r="B29" s="38" t="inlineStr">
         <is>
           <t>Louis Toffoli</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C29" s="38" t="inlineStr">
         <is>
           <t>Annonces particuliers et galeries</t>
         </is>
       </c>
-      <c r="D8" s="33" t="inlineStr">
+      <c r="D29" s="38" t="inlineStr">
         <is>
           <t>PRIX DEMANDÉ</t>
         </is>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E29" s="39" t="n">
         <v>120</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F29" s="39" t="n">
         <v>1090</v>
       </c>
-      <c r="G8" s="33" t="inlineStr">
+      <c r="G29" s="38" t="inlineStr">
         <is>
           <t>leboncoin, eBay, passion-estampes</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t>Claude Weisbuch</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>« Grande parade », litho signée BD</t>
-        </is>
-      </c>
-      <c r="D9" s="31" t="inlineStr">
-        <is>
-          <t>Estimation salle (2025)</t>
-        </is>
-      </c>
-      <c r="E9" s="32" t="n">
-        <v>200</v>
-      </c>
-      <c r="F9" s="32" t="n">
-        <v>300</v>
-      </c>
-      <c r="G9" s="31" t="inlineStr">
-        <is>
-          <t>primardeco.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>Claude Weisbuch</t>
-        </is>
-      </c>
-      <c r="C10" s="29" t="inlineStr">
-        <is>
-          <t>Fourchette générale des multiples</t>
-        </is>
-      </c>
-      <c r="D10" s="29" t="inlineStr">
-        <is>
-          <t>Adjugé (marché)</t>
-        </is>
-      </c>
-      <c r="E10" s="30" t="n">
-        <v>30</v>
-      </c>
-      <c r="F10" s="30" t="n">
-        <v>400</v>
-      </c>
-      <c r="G10" s="29" t="inlineStr">
-        <is>
-          <t>mr-expert.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="33" t="inlineStr">
-        <is>
-          <t>Claude Weisbuch</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="inlineStr">
-        <is>
-          <t>« Deux Cavaliers », litho signée /125</t>
-        </is>
-      </c>
-      <c r="D11" s="33" t="inlineStr">
-        <is>
-          <t>PRIX DEMANDÉ</t>
-        </is>
-      </c>
-      <c r="E11" s="34" t="n">
-        <v>487</v>
-      </c>
-      <c r="F11" s="34" t="n">
-        <v>487</v>
-      </c>
-      <c r="G11" s="33" t="inlineStr">
-        <is>
-          <t>1stdibs.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Artprice : outil de recherche, PAS un canal de vente</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="n"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Ce que c'est</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Une base de 30 millions de résultats d'enchères sur 700 000 artistes. C'est l'outil que les commissaires-priseurs consultent pour estimer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Le coût</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Abonnement obligatoire : 196 €/an en basique, jusqu'à 407 €/an en pro. Sa marketplace prend en plus 5 à 9 % TTC de frais vendeur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Le problème</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>L'audience y vient CHERCHER DES PRIX, pas acheter de la décoration murale. Pour écouler 300 lithographies d'éditeur, le débit est quasi nul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Ne t'abonne pas pour vendre. Si tu veux des résultats d'enchères, Interencheres, Gazette Drouot, Barnebys et le filtre « objets vendus » d'eBay te donnent l'essentiel gratuitement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Ce que disent les experts du marché</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="B14" s="5" t="inlineStr">
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>Toffoli</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>« Très nombreuses sur le marché de l'art, la réelle valeur des estampes est aujourd'hui très faible. » — expertisez.com</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="B15" s="5" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Weisbuch</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>« La cote subit une tendance à la baisse et une désaffection des acquéreurs, car les estimations trop élevées ne trouvent pas d'acheteurs. » — mr-expert.com</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Conséquence</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Le prix affiché n'est pas le problème : c'est le prix auquel un acheteur clique. Vise le haut de la fourchette ADJUGÉE, pas le bas de la fourchette DEMANDÉE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="3" t="inlineStr">
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Hilaire</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Marché stable mais encombré : la plupart des lithos signées se négocient entre 89 et 150 €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Brayer</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Le seul dont les séries complètes atteignent 1 000 à 2 000 €. Ne casse jamais une suite pour la vendre à la pièce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>Ce qui fait monter le prix</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>•  Petit tirage (moins de 150) plutôt que 250-300.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>•  Sujet recherché : musiciens, maternités, marines, travailleurs pour Toffoli ; cavaliers, musiciens, théâtre pour Weisbuch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="4" t="inlineStr">
+    <row r="45" ht="26" customHeight="1">
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>•  Sujet recherché : Camargue, taureaux et Provence pour Brayer ; cavaliers, musiciens et théâtre pour Weisbuch ; musiciens, maternités et marines pour Toffoli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>•  Épreuve d'artiste (EA) ou hors commerce (HC) plutôt qu'un simple numéro.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>•  Vraie lithographie sur pierre (grain irrégulier) plutôt qu'un offset signé.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="C24" s="4" t="inlineStr">
+    <row r="47" ht="26" customHeight="1">
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>•  Suite ou portfolio complet gardé groupé — chez Brayer, ça double la mise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>•  Papier de qualité à bords barbés (Arches, BFK Rives) + timbre sec d'atelier.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>•  État neuf, marges intactes, jamais encadré sous verre sans marie-louise.</t>
+    <row r="49" ht="26" customHeight="1">
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>•  État neuf, marges intactes, jamais massicotées.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="C22:G22"/>
+  <mergeCells count="20">
+    <mergeCell ref="C49:G49"/>
+    <mergeCell ref="C34:G34"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="C33:G33"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="C45:G45"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C47:G47"/>
+    <mergeCell ref="C44:G44"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="C46:G46"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="C48:G48"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="B11:G11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17313,206 +17826,206 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="35" t="inlineStr">
+      <c r="B4" s="40" t="inlineStr">
         <is>
           <t>Période</t>
         </is>
       </c>
-      <c r="C4" s="35" t="inlineStr">
+      <c r="C4" s="40" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D4" s="35" t="inlineStr">
+      <c r="D4" s="40" t="inlineStr">
         <is>
           <t>Détail</t>
         </is>
       </c>
-      <c r="E4" s="35" t="inlineStr">
+      <c r="E4" s="40" t="inlineStr">
         <is>
           <t>Fait ?</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="41" t="inlineStr">
         <is>
           <t>Semaines 1-3</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="32" t="inlineStr">
         <is>
           <t>Inventaire complet</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="D5" s="32" t="inlineStr">
         <is>
           <t>Photographier et saisir les 300 pièces. 20 par séance. Pour chaque : vue entière + macro de la signature + macro de la numérotation. Fond blanc, lumière du jour, pas de flash.</t>
         </is>
       </c>
-      <c r="E5" s="36" t="inlineStr"/>
+      <c r="E5" s="42" t="inlineStr"/>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr">
         <is>
           <t>Semaine 2</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="32" t="inlineStr">
         <is>
           <t>Test loupe x10</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D6" s="32" t="inlineStr">
         <is>
           <t>Sur 10 pièces représentatives : grain irrégulier = vraie litho ; trame de points réguliers = offset. Décide du vocabulaire de tes annonces en conséquence.</t>
         </is>
       </c>
-      <c r="E6" s="36" t="inlineStr"/>
+      <c r="E6" s="42" t="inlineStr"/>
     </row>
     <row r="7" ht="46" customHeight="1">
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>Semaine 3</t>
         </is>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>Identifier les artistes manquants</t>
         </is>
       </c>
-      <c r="D7" s="31" t="inlineStr">
+      <c r="D7" s="32" t="inlineStr">
         <is>
           <t>Photo macro de chaque signature illisible. Recouper avec les certificats d'authenticité et les bons de livraison de l'éditeur.</t>
         </is>
       </c>
-      <c r="E7" s="36" t="inlineStr"/>
+      <c r="E7" s="42" t="inlineStr"/>
     </row>
     <row r="8" ht="46" customHeight="1">
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>Semaine 4</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
         <is>
           <t>Segmentation A / B / C</t>
         </is>
       </c>
-      <c r="D8" s="31" t="inlineStr">
+      <c r="D8" s="32" t="inlineStr">
         <is>
           <t>Croiser artiste + sujet + tirage + doubles. Vise environ 15 % en A, 45 % en B, 40 % en C.</t>
         </is>
       </c>
-      <c r="E8" s="36" t="inlineStr"/>
+      <c r="E8" s="42" t="inlineStr"/>
     </row>
     <row r="9" ht="46" customHeight="1">
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr">
         <is>
           <t>Semaines 5-8</t>
         </is>
       </c>
-      <c r="C9" s="31" t="inlineStr">
+      <c r="C9" s="32" t="inlineStr">
         <is>
           <t>Test de marché</t>
         </is>
       </c>
-      <c r="D9" s="31" t="inlineStr">
+      <c r="D9" s="32" t="inlineStr">
         <is>
           <t>Mettre en vente 8 à 10 pièces seulement : 3 en enchères (Drouot Online / Interencheres), 3 sur eBay au prix cible, 3 sur Le Bon Coin en remise en main propre Paris. Noter les prix obtenus.</t>
         </is>
       </c>
-      <c r="E9" s="36" t="inlineStr"/>
+      <c r="E9" s="42" t="inlineStr"/>
     </row>
     <row r="10" ht="46" customHeight="1">
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="41" t="inlineStr">
         <is>
           <t>Semaine 9</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="32" t="inlineStr">
         <is>
           <t>Recalibrer</t>
         </is>
       </c>
-      <c r="D10" s="31" t="inlineStr">
+      <c r="D10" s="32" t="inlineStr">
         <is>
           <t>Réviser tous les prix cibles à partir des résultats réels. C'est ici que le tableau de bord sert.</t>
         </is>
       </c>
-      <c r="E10" s="36" t="inlineStr"/>
+      <c r="E10" s="42" t="inlineStr"/>
     </row>
     <row r="11" ht="46" customHeight="1">
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
         <is>
           <t>Mois 3-12</t>
         </is>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="32" t="inlineStr">
         <is>
           <t>Écoulement du segment A puis B</t>
         </is>
       </c>
-      <c r="D11" s="31" t="inlineStr">
+      <c r="D11" s="32" t="inlineStr">
         <is>
           <t>5 à 10 annonces actives en permanence, jamais deux fois la même image. Renouveler chaque pièce vendue.</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr"/>
+      <c r="E11" s="42" t="inlineStr"/>
     </row>
     <row r="12" ht="46" customHeight="1">
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
         <is>
           <t>Mois 3-24</t>
         </is>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
         <is>
           <t>Segment C en lots</t>
         </is>
       </c>
-      <c r="D12" s="31" t="inlineStr">
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>Lots thématiques de 5 à 20 sur eBay/Catawiki, ou cession en bloc à un marchand (compter 20-30 % du prix de détail, mais tout part d'un coup).</t>
         </is>
       </c>
-      <c r="E12" s="36" t="inlineStr"/>
+      <c r="E12" s="42" t="inlineStr"/>
     </row>
     <row r="13" ht="46" customHeight="1">
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="41" t="inlineStr">
         <is>
           <t>En parallèle</t>
         </is>
       </c>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>Consignation en salle</t>
         </is>
       </c>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="D13" s="32" t="inlineStr">
         <is>
           <t>Prendre rendez-vous avec 2-3 maisons parisiennes (Drouot, Millon, Lucien Paris, Richard). Estimation gratuite. Leur confier des lots groupés d'artistes secondaires.</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr"/>
+      <c r="E13" s="42" t="inlineStr"/>
     </row>
     <row r="14" ht="46" customHeight="1">
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="41" t="inlineStr">
         <is>
           <t>En continu</t>
         </is>
       </c>
-      <c r="C14" s="31" t="inlineStr">
+      <c r="C14" s="32" t="inlineStr">
         <is>
           <t>Logistique</t>
         </is>
       </c>
-      <c r="D14" s="31" t="inlineStr">
+      <c r="D14" s="32" t="inlineStr">
         <is>
           <t>Tubes rigides Ø10 cm et pochettes cristal. Pour du 56x76, la remise en main propre à Paris évite 15-25 € de port et les litiges pour pliure — privilégie-la.</t>
         </is>
       </c>
-      <c r="E14" s="36" t="inlineStr"/>
+      <c r="E14" s="42" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
@@ -17544,154 +18057,154 @@
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="B19" s="31" t="inlineStr">
+      <c r="B19" s="32" t="inlineStr">
         <is>
           <t>Le Bon Coin (Paris)</t>
         </is>
       </c>
-      <c r="C19" s="31" t="inlineStr">
+      <c r="C19" s="32" t="inlineStr">
         <is>
           <t>0 %</t>
         </is>
       </c>
-      <c r="D19" s="31" t="inlineStr">
+      <c r="D19" s="32" t="inlineStr">
         <is>
           <t>Rapide, main propre, zéro port</t>
         </is>
       </c>
-      <c r="E19" s="31" t="inlineStr">
+      <c r="E19" s="32" t="inlineStr">
         <is>
           <t>A et B — le meilleur rapport effort/net pour du 56x76</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="B20" s="31" t="inlineStr">
+      <c r="B20" s="32" t="inlineStr">
         <is>
           <t>eBay</t>
         </is>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="32" t="inlineStr">
         <is>
           <t>~12 % + port</t>
         </is>
       </c>
-      <c r="D20" s="31" t="inlineStr">
+      <c r="D20" s="32" t="inlineStr">
         <is>
           <t>Moyen, audience large</t>
         </is>
       </c>
-      <c r="E20" s="31" t="inlineStr">
+      <c r="E20" s="32" t="inlineStr">
         <is>
           <t>A et B, et lots du segment C</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="31" t="inlineStr">
+      <c r="B21" s="32" t="inlineStr">
         <is>
           <t>Catawiki</t>
         </is>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C21" s="32" t="inlineStr">
         <is>
           <t>~12,5 % vendeur</t>
         </is>
       </c>
-      <c r="D21" s="31" t="inlineStr">
+      <c r="D21" s="32" t="inlineStr">
         <is>
           <t>Lent (sélection), acheteurs internationaux</t>
         </is>
       </c>
-      <c r="E21" s="31" t="inlineStr">
+      <c r="E21" s="32" t="inlineStr">
         <is>
           <t>A surtout — met en valeur les belles pièces</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="31" t="inlineStr">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>Enchères en salle</t>
         </is>
       </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="C22" s="32" t="inlineStr">
         <is>
           <t>15-25 % + frais</t>
         </is>
       </c>
-      <c r="D22" s="31" t="inlineStr">
+      <c r="D22" s="32" t="inlineStr">
         <is>
           <t>Aucun effort, mais prix bas et invendus</t>
         </is>
       </c>
-      <c r="E22" s="31" t="inlineStr">
+      <c r="E22" s="32" t="inlineStr">
         <is>
           <t>C et doubles, ou test de marché</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="31" t="inlineStr">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t>Marchand en gros</t>
         </is>
       </c>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C23" s="32" t="inlineStr">
         <is>
           <t>20-30 % du détail</t>
         </is>
       </c>
-      <c r="D23" s="31" t="inlineStr">
+      <c r="D23" s="32" t="inlineStr">
         <is>
           <t>Immédiat, tout part</t>
         </is>
       </c>
-      <c r="E23" s="31" t="inlineStr">
+      <c r="E23" s="32" t="inlineStr">
         <is>
           <t>C — la queue de collection</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="B24" s="31" t="inlineStr">
+      <c r="B24" s="32" t="inlineStr">
         <is>
           <t>Etsy</t>
         </is>
       </c>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="C24" s="32" t="inlineStr">
         <is>
           <t>~9 % + port</t>
         </is>
       </c>
-      <c r="D24" s="31" t="inlineStr">
+      <c r="D24" s="32" t="inlineStr">
         <is>
           <t>Lent, marché déco international</t>
         </is>
       </c>
-      <c r="E24" s="31" t="inlineStr">
+      <c r="E24" s="32" t="inlineStr">
         <is>
           <t>B, sujets décoratifs</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="B25" s="31" t="inlineStr">
+      <c r="B25" s="32" t="inlineStr">
         <is>
           <t>Galerie en dépôt-vente</t>
         </is>
       </c>
-      <c r="C25" s="31" t="inlineStr">
+      <c r="C25" s="32" t="inlineStr">
         <is>
           <t>30-50 %</t>
         </is>
       </c>
-      <c r="D25" s="31" t="inlineStr">
+      <c r="D25" s="32" t="inlineStr">
         <is>
           <t>Très lent</t>
         </is>
       </c>
-      <c r="E25" s="31" t="inlineStr">
+      <c r="E25" s="32" t="inlineStr">
         <is>
           <t>A uniquement, si la galerie est spécialisée estampe</t>
         </is>

</xml_diff>